<commit_message>
Added a terminal block footprint, 3d model, and updated database
</commit_message>
<xml_diff>
--- a/To Add v2/Connectors - Terminal Blocks - Wire to Board.xlsx
+++ b/To Add v2/Connectors - Terminal Blocks - Wire to Board.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\To Add v2\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Github\Danakil_KiCad_DB\To Add v2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2122E87E-2E72-42C8-8E8C-CEA37E6FA15E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55965057-FE9F-43A7-88C6-4EF04BDB7D46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2304" yWindow="1452" windowWidth="18732" windowHeight="11508" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="7725" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="445" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="445" uniqueCount="126">
   <si>
     <t>Totals</t>
   </si>
@@ -411,6 +411,9 @@
   </si>
   <si>
     <t>0Dan_Connectors:Conn_01x16</t>
+  </si>
+  <si>
+    <t>TermBlocks:691137710004</t>
   </si>
 </sst>
 </file>
@@ -766,27 +769,27 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AC166"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="3" max="3" width="56" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.21875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5546875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="9.77734375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="9.77734375" customWidth="1"/>
-    <col min="14" max="14" width="14.77734375" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="21.109375" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="12.109375" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="25.6640625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="31.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="29.1796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.54296875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="9.81640625" customWidth="1"/>
+    <col min="14" max="14" width="14.81640625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="21.08984375" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="9.6328125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="12.08984375" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="25.6328125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="31.08984375" bestFit="1" customWidth="1"/>
     <col min="28" max="28" width="15" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:29" x14ac:dyDescent="0.35">
       <c r="B1" s="1"/>
       <c r="O1" s="1"/>
     </row>
-    <row r="2" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:29" x14ac:dyDescent="0.35">
       <c r="B2" t="s">
         <v>0</v>
       </c>
@@ -874,7 +877,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="3" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:29" x14ac:dyDescent="0.35">
       <c r="AB3" t="s">
         <v>2</v>
       </c>
@@ -883,7 +886,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="4" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:29" x14ac:dyDescent="0.35">
       <c r="B4" t="s">
         <v>3</v>
       </c>
@@ -952,7 +955,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="5" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:29" x14ac:dyDescent="0.35">
       <c r="AB5" t="s">
         <v>5</v>
       </c>
@@ -961,7 +964,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:29" x14ac:dyDescent="0.35">
       <c r="C6" t="s">
         <v>6</v>
       </c>
@@ -1029,7 +1032,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="7" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>1</v>
       </c>
@@ -1112,7 +1115,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="8" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>2</v>
       </c>
@@ -1188,13 +1191,13 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>3</v>
       </c>
       <c r="C9" t="str">
         <f t="shared" si="3"/>
-        <v>4Pos WR-TBL_1377 Horiz Screw 300v 16A 5mm 12-30AWG Green No_FP</v>
+        <v>4Pos WR-TBL_1377 Horiz Screw 300v 16A 5mm 12-30AWG Green  </v>
       </c>
       <c r="D9" t="str">
         <f t="shared" si="4"/>
@@ -1246,10 +1249,10 @@
         <v>117</v>
       </c>
       <c r="T9" t="s">
+        <v>125</v>
+      </c>
+      <c r="U9" t="s">
         <v>108</v>
-      </c>
-      <c r="U9" t="s">
-        <v>109</v>
       </c>
       <c r="X9">
         <f t="shared" si="5"/>
@@ -1264,7 +1267,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>4</v>
       </c>
@@ -1340,7 +1343,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>5</v>
       </c>
@@ -1416,7 +1419,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>6</v>
       </c>
@@ -1492,7 +1495,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>7</v>
       </c>
@@ -1568,7 +1571,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>8</v>
       </c>
@@ -1644,7 +1647,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>9</v>
       </c>
@@ -1720,7 +1723,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A16">
         <v>10</v>
       </c>
@@ -1796,7 +1799,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>11</v>
       </c>
@@ -1872,7 +1875,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>12</v>
       </c>
@@ -1948,7 +1951,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>13</v>
       </c>
@@ -2024,7 +2027,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>14</v>
       </c>
@@ -2100,7 +2103,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A21">
         <v>15</v>
       </c>
@@ -2176,7 +2179,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A22">
         <v>16</v>
       </c>
@@ -2252,7 +2255,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A23">
         <v>17</v>
       </c>
@@ -2328,7 +2331,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A24">
         <v>18</v>
       </c>
@@ -2404,7 +2407,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A25">
         <v>19</v>
       </c>
@@ -2480,7 +2483,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A26">
         <v>20</v>
       </c>
@@ -2556,7 +2559,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A27">
         <v>21</v>
       </c>
@@ -2632,7 +2635,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A28">
         <v>22</v>
       </c>
@@ -2708,7 +2711,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A29">
         <v>23</v>
       </c>
@@ -2784,7 +2787,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A30">
         <v>24</v>
       </c>
@@ -2860,7 +2863,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A31">
         <v>25</v>
       </c>
@@ -2936,7 +2939,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A32">
         <v>26</v>
       </c>
@@ -3012,406 +3015,406 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="33" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O33" s="2"/>
     </row>
-    <row r="34" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="34" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O34" s="2"/>
     </row>
-    <row r="35" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="35" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O35" s="2"/>
     </row>
-    <row r="36" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="36" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O36" s="2"/>
     </row>
-    <row r="37" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="37" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O37" s="2"/>
     </row>
-    <row r="38" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="38" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O38" s="2"/>
     </row>
-    <row r="39" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="39" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O39" s="2"/>
     </row>
-    <row r="40" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="40" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O40" s="2"/>
     </row>
-    <row r="41" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="41" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O41" s="2"/>
     </row>
-    <row r="42" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="42" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O42" s="2"/>
     </row>
-    <row r="43" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="43" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O43" s="2"/>
     </row>
-    <row r="44" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="44" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O44" s="2"/>
     </row>
-    <row r="45" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="45" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O45" s="2"/>
     </row>
-    <row r="46" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="46" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O46" s="2"/>
     </row>
-    <row r="47" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="47" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O47" s="2"/>
     </row>
-    <row r="48" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="48" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O48" s="2"/>
     </row>
-    <row r="49" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="49" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O49" s="2"/>
     </row>
-    <row r="50" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="50" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O50" s="2"/>
     </row>
-    <row r="51" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="51" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O51" s="2"/>
     </row>
-    <row r="52" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="52" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O52" s="2"/>
     </row>
-    <row r="53" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="53" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O53" s="2"/>
     </row>
-    <row r="54" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="54" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O54" s="2"/>
     </row>
-    <row r="55" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="55" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O55" s="2"/>
     </row>
-    <row r="56" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="56" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O56" s="2"/>
     </row>
-    <row r="57" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="57" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O57" s="2"/>
     </row>
-    <row r="58" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="58" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O58" s="2"/>
     </row>
-    <row r="59" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="59" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O59" s="2"/>
     </row>
-    <row r="60" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="60" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O60" s="2"/>
     </row>
-    <row r="61" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="61" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O61" s="2"/>
     </row>
-    <row r="62" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="62" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O62" s="2"/>
     </row>
-    <row r="63" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="63" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O63" s="2"/>
     </row>
-    <row r="64" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="64" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O64" s="2"/>
     </row>
-    <row r="65" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="65" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O65" s="2"/>
     </row>
-    <row r="66" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="66" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O66" s="2"/>
     </row>
-    <row r="67" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="67" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O67" s="2"/>
     </row>
-    <row r="68" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="68" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O68" s="2"/>
     </row>
-    <row r="69" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="69" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O69" s="2"/>
     </row>
-    <row r="70" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="70" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O70" s="2"/>
     </row>
-    <row r="71" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="71" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O71" s="2"/>
     </row>
-    <row r="72" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="72" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O72" s="2"/>
     </row>
-    <row r="73" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="73" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O73" s="2"/>
     </row>
-    <row r="74" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="74" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O74" s="2"/>
     </row>
-    <row r="75" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="75" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O75" s="2"/>
     </row>
-    <row r="76" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="76" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O76" s="2"/>
     </row>
-    <row r="77" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="77" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O77" s="2"/>
     </row>
-    <row r="78" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="78" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O78" s="2"/>
     </row>
-    <row r="79" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="79" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O79" s="2"/>
     </row>
-    <row r="80" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="80" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O80" s="2"/>
     </row>
-    <row r="81" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="81" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O81" s="2"/>
     </row>
-    <row r="82" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="82" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O82" s="2"/>
     </row>
-    <row r="83" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="83" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O83" s="2"/>
     </row>
-    <row r="84" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="84" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O84" s="2"/>
     </row>
-    <row r="85" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="85" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O85" s="2"/>
     </row>
-    <row r="86" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="86" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O86" s="2"/>
     </row>
-    <row r="87" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="87" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O87" s="2"/>
     </row>
-    <row r="88" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="88" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O88" s="2"/>
     </row>
-    <row r="89" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="89" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O89" s="2"/>
     </row>
-    <row r="90" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="90" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O90" s="2"/>
     </row>
-    <row r="91" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="91" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O91" s="2"/>
     </row>
-    <row r="92" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="92" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O92" s="2"/>
     </row>
-    <row r="93" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="93" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O93" s="2"/>
     </row>
-    <row r="94" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="94" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O94" s="2"/>
     </row>
-    <row r="95" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="95" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O95" s="2"/>
     </row>
-    <row r="96" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="96" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O96" s="2"/>
     </row>
-    <row r="97" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="97" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O97" s="2"/>
     </row>
-    <row r="98" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="98" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O98" s="2"/>
     </row>
-    <row r="99" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="99" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O99" s="2"/>
     </row>
-    <row r="100" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="100" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O100" s="2"/>
     </row>
-    <row r="101" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="101" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O101" s="2"/>
     </row>
-    <row r="102" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="102" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O102" s="2"/>
     </row>
-    <row r="103" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="103" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O103" s="2"/>
     </row>
-    <row r="104" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="104" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O104" s="2"/>
     </row>
-    <row r="105" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="105" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O105" s="2"/>
     </row>
-    <row r="106" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="106" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O106" s="2"/>
     </row>
-    <row r="107" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="107" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O107" s="2"/>
     </row>
-    <row r="108" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="108" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O108" s="2"/>
     </row>
-    <row r="109" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="109" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O109" s="2"/>
     </row>
-    <row r="110" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="110" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O110" s="2"/>
     </row>
-    <row r="111" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="111" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O111" s="2"/>
     </row>
-    <row r="112" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="112" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O112" s="2"/>
     </row>
-    <row r="113" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="113" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O113" s="2"/>
     </row>
-    <row r="114" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="114" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O114" s="2"/>
     </row>
-    <row r="115" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="115" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O115" s="2"/>
     </row>
-    <row r="116" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="116" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O116" s="2"/>
     </row>
-    <row r="117" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="117" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O117" s="2"/>
     </row>
-    <row r="118" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="118" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O118" s="2"/>
     </row>
-    <row r="119" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="119" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O119" s="2"/>
     </row>
-    <row r="120" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="120" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O120" s="2"/>
     </row>
-    <row r="121" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="121" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O121" s="2"/>
     </row>
-    <row r="122" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="122" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O122" s="2"/>
     </row>
-    <row r="123" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="123" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O123" s="2"/>
     </row>
-    <row r="124" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="124" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O124" s="2"/>
     </row>
-    <row r="125" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="125" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O125" s="2"/>
     </row>
-    <row r="126" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="126" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O126" s="2"/>
     </row>
-    <row r="127" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="127" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O127" s="2"/>
     </row>
-    <row r="128" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="128" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O128" s="2"/>
     </row>
-    <row r="129" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="129" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O129" s="2"/>
     </row>
-    <row r="130" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="130" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O130" s="2"/>
     </row>
-    <row r="131" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="131" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O131" s="2"/>
     </row>
-    <row r="132" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="132" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O132" s="2"/>
     </row>
-    <row r="133" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="133" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O133" s="2"/>
     </row>
-    <row r="134" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="134" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O134" s="2"/>
     </row>
-    <row r="135" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="135" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O135" s="2"/>
     </row>
-    <row r="136" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="136" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O136" s="2"/>
     </row>
-    <row r="137" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="137" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O137" s="2"/>
     </row>
-    <row r="138" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="138" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O138" s="2"/>
     </row>
-    <row r="139" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="139" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O139" s="2"/>
     </row>
-    <row r="140" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="140" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O140" s="2"/>
     </row>
-    <row r="141" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="141" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O141" s="2"/>
     </row>
-    <row r="142" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="142" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O142" s="2"/>
     </row>
-    <row r="143" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="143" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O143" s="2"/>
     </row>
-    <row r="144" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="144" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O144" s="2"/>
     </row>
-    <row r="145" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="145" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O145" s="2"/>
     </row>
-    <row r="146" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="146" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O146" s="2"/>
     </row>
-    <row r="147" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="147" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O147" s="2"/>
     </row>
-    <row r="148" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="148" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O148" s="2"/>
     </row>
-    <row r="149" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="149" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O149" s="2"/>
     </row>
-    <row r="150" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="150" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O150" s="2"/>
     </row>
-    <row r="151" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="151" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O151" s="2"/>
     </row>
-    <row r="152" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="152" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O152" s="2"/>
     </row>
-    <row r="153" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="153" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O153" s="2"/>
     </row>
-    <row r="154" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="154" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O154" s="2"/>
     </row>
-    <row r="155" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="155" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O155" s="2"/>
     </row>
-    <row r="156" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="156" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O156" s="2"/>
     </row>
-    <row r="157" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="157" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O157" s="2"/>
     </row>
-    <row r="158" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="158" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O158" s="2"/>
     </row>
-    <row r="159" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="159" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O159" s="2"/>
     </row>
-    <row r="160" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="160" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O160" s="2"/>
     </row>
-    <row r="161" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="161" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O161" s="2"/>
     </row>
-    <row r="162" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="162" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O162" s="2"/>
     </row>
-    <row r="163" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="163" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O163" s="2"/>
     </row>
-    <row r="164" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="164" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O164" s="2"/>
     </row>
-    <row r="165" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="165" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O165" s="2"/>
     </row>
-    <row r="166" spans="15:15" x14ac:dyDescent="0.3">
+    <row r="166" spans="15:15" x14ac:dyDescent="0.35">
       <c r="O166" s="2"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added a 5 pos terminal block footprint, model, and updated database
</commit_message>
<xml_diff>
--- a/To Add v2/Connectors - Terminal Blocks - Wire to Board.xlsx
+++ b/To Add v2/Connectors - Terminal Blocks - Wire to Board.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Github\Danakil_KiCad_DB\To Add v2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55965057-FE9F-43A7-88C6-4EF04BDB7D46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06C91556-DCA5-4DBE-BB5D-FF9CD0B5EF2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="7725" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="445" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="445" uniqueCount="127">
   <si>
     <t>Totals</t>
   </si>
@@ -414,6 +414,9 @@
   </si>
   <si>
     <t>TermBlocks:691137710004</t>
+  </si>
+  <si>
+    <t>TermBlocks:TB002-500-05BE</t>
   </si>
 </sst>
 </file>
@@ -1501,7 +1504,7 @@
       </c>
       <c r="C13" t="str">
         <f t="shared" si="3"/>
-        <v>5Pos TB002-500 Horiz Screw 300v 15A 5mm 12-22AWG Cyan No_FP</v>
+        <v>5Pos TB002-500 Horiz Screw 300v 15A 5mm 12-22AWG Cyan  </v>
       </c>
       <c r="D13" t="str">
         <f t="shared" si="4"/>
@@ -1553,10 +1556,10 @@
         <v>118</v>
       </c>
       <c r="T13" t="s">
+        <v>126</v>
+      </c>
+      <c r="U13" t="s">
         <v>108</v>
-      </c>
-      <c r="U13" t="s">
-        <v>109</v>
       </c>
       <c r="X13">
         <f t="shared" si="5"/>

</xml_diff>